<commit_message>
add board design link
</commit_message>
<xml_diff>
--- a/ESP32-S2-REV-TFT/EncLickDrv_J0104132C-ESPrevC.xlsx
+++ b/ESP32-S2-REV-TFT/EncLickDrv_J0104132C-ESPrevC.xlsx
@@ -8,19 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sawtelles\Documents\GitHub\Treadmill-Interface\ESP32-S2-REV-TFT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36C8B260-B4F0-4872-896E-166C444728FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1DEDC89-9956-4430-8F3A-8311D1750CE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="18240" windowHeight="28320" xr2:uid="{416FB7B0-818F-482A-B6F8-C23829542AFB}"/>
   </bookViews>
   <sheets>
     <sheet name="EncLickDrv_J0104132C-ESPrevB" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="81">
   <si>
     <t>Partlist exported from Z:/ID&amp;F/TreadmillWithLick/EncoderLickDriver/ECAD/EncLickDrv_J0104132C-ESPrevB.sch at 7/21/2025 11:48 AM</t>
   </si>
@@ -254,6 +267,15 @@
   </si>
   <si>
     <t>900-0530480560-ND</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
+  </si>
+  <si>
+    <t>BOARD design can be found at:</t>
+  </si>
+  <si>
+    <t>https://oshpark.com/shared_projects/oZUU0shd</t>
   </si>
 </sst>
 </file>
@@ -1125,7 +1147,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E29F0A2C-E311-4CCC-8F5B-171C8FA56A01}">
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="25" customWidth="1"/>
@@ -1134,6 +1156,7 @@
     <col min="5" max="5" width="15.28515625" customWidth="1"/>
     <col min="6" max="6" width="17.85546875" customWidth="1"/>
     <col min="8" max="8" width="20.7109375" customWidth="1"/>
+    <col min="9" max="9" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -1166,7 +1189,7 @@
       <c r="H3" t="s">
         <v>8</v>
       </c>
-      <c r="I3" t="s">
+      <c r="I3" s="1" t="s">
         <v>9</v>
       </c>
       <c r="J3" t="s">
@@ -1545,6 +1568,25 @@
       </c>
       <c r="I19" s="1">
         <v>2.8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="H21" t="s">
+        <v>78</v>
+      </c>
+      <c r="I21" s="1">
+        <f>SUM(I4:I20)</f>
+        <v>44.999999999999993</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C22" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C23" t="s">
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update readme, add license file
</commit_message>
<xml_diff>
--- a/ESP32-S2-REV-TFT/EncLickDrv_J0104132C-ESPrevC.xlsx
+++ b/ESP32-S2-REV-TFT/EncLickDrv_J0104132C-ESPrevC.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sawtelles\Documents\GitHub\Treadmill-Interface\ESP32-S2-REV-TFT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1DEDC89-9956-4430-8F3A-8311D1750CE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7450101B-4A80-48A1-A0F8-2C4A12CC7C01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="18240" windowHeight="28320" xr2:uid="{416FB7B0-818F-482A-B6F8-C23829542AFB}"/>
+    <workbookView xWindow="7590" yWindow="540" windowWidth="25215" windowHeight="14850" xr2:uid="{416FB7B0-818F-482A-B6F8-C23829542AFB}"/>
   </bookViews>
   <sheets>
     <sheet name="EncLickDrv_J0104132C-ESPrevB" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="86">
   <si>
     <t>Partlist exported from Z:/ID&amp;F/TreadmillWithLick/EncoderLickDriver/ECAD/EncLickDrv_J0104132C-ESPrevB.sch at 7/21/2025 11:48 AM</t>
   </si>
@@ -276,6 +276,21 @@
   </si>
   <si>
     <t>https://oshpark.com/shared_projects/oZUU0shd</t>
+  </si>
+  <si>
+    <t>Alternate</t>
+  </si>
+  <si>
+    <t>CONN HEADER R/A 5POS 2.54MM</t>
+  </si>
+  <si>
+    <t>5-104361-4</t>
+  </si>
+  <si>
+    <t>A33964-ND</t>
+  </si>
+  <si>
+    <t>5 pin header RA</t>
   </si>
 </sst>
 </file>
@@ -1504,7 +1519,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>1</v>
       </c>
@@ -1527,7 +1542,7 @@
         <v>2.62</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2</v>
       </c>
@@ -1556,7 +1571,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C19" t="s">
         <v>63</v>
       </c>
@@ -1570,21 +1585,53 @@
         <v>2.8</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>1</v>
+      </c>
+      <c r="B20" t="s">
+        <v>85</v>
+      </c>
+      <c r="C20" t="s">
+        <v>82</v>
+      </c>
+      <c r="D20" t="s">
+        <v>34</v>
+      </c>
+      <c r="E20" t="s">
+        <v>61</v>
+      </c>
+      <c r="F20" t="s">
+        <v>83</v>
+      </c>
+      <c r="G20" t="s">
+        <v>46</v>
+      </c>
+      <c r="H20" t="s">
+        <v>84</v>
+      </c>
+      <c r="I20" s="1">
+        <v>1.74</v>
+      </c>
+      <c r="J20" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H21" t="s">
         <v>78</v>
       </c>
       <c r="I21" s="1">
         <f>SUM(I4:I20)</f>
-        <v>44.999999999999993</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+        <v>46.739999999999995</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C22" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C23" t="s">
         <v>80</v>
       </c>

</xml_diff>